<commit_message>
Add clock, unit filter, and employee detail cards to dashboard
- Header shows a live clock next to the date, ticked every 30s and
  rendered client-side to avoid an SSR mismatch.
- Locations become three units: Noida, Gurgaon, Okhla. Credentials
  sheet regenerated to match.
- Manager dashboard: swap the open-issues tile for tasks pending, add
  a unit filter, and replace the detail table with employee cards that
  turn green at 100% and open a modal with per-task tick times.
- Drop the completion-by-employee bars and their now-dead CSS.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/credentials.xlsx
+++ b/public/credentials.xlsx
@@ -437,7 +437,7 @@
         <v>Manager@123</v>
       </c>
       <c r="E2" t="str">
-        <v>All locations</v>
+        <v>All units</v>
       </c>
     </row>
     <row r="3">
@@ -454,7 +454,7 @@
         <v>Amit@123</v>
       </c>
       <c r="E3" t="str">
-        <v>Downtown Hub</v>
+        <v>Noida</v>
       </c>
     </row>
     <row r="4">
@@ -471,7 +471,7 @@
         <v>Priya@123</v>
       </c>
       <c r="E4" t="str">
-        <v>Downtown Hub</v>
+        <v>Noida</v>
       </c>
     </row>
     <row r="5">
@@ -488,7 +488,7 @@
         <v>Rahul@123</v>
       </c>
       <c r="E5" t="str">
-        <v>Riverside</v>
+        <v>Gurgaon</v>
       </c>
     </row>
     <row r="6">
@@ -505,7 +505,7 @@
         <v>Sara@123</v>
       </c>
       <c r="E6" t="str">
-        <v>Uptown Central</v>
+        <v>Gurgaon</v>
       </c>
     </row>
     <row r="7">
@@ -522,7 +522,7 @@
         <v>John@123</v>
       </c>
       <c r="E7" t="str">
-        <v>Lakeside</v>
+        <v>Okhla</v>
       </c>
     </row>
     <row r="8">
@@ -539,7 +539,7 @@
         <v>Meera@123</v>
       </c>
       <c r="E8" t="str">
-        <v>Tech Park</v>
+        <v>Okhla</v>
       </c>
     </row>
   </sheetData>

</xml_diff>